<commit_message>
Update notification list, add email list template, and update logs
</commit_message>
<xml_diff>
--- a/bdays.xlsx
+++ b/bdays.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="89">
   <si>
     <t>Name</t>
   </si>
@@ -51,20 +51,245 @@
     <t>alfredsam2006@gmail.com</t>
   </si>
   <si>
-    <t>hippy</t>
-  </si>
-  <si>
     <t>alfredsam427@gmail.com</t>
   </si>
   <si>
-    <t>06-15-2006</t>
+    <t>Bharathwaj S</t>
+  </si>
+  <si>
+    <t>Darshan S</t>
+  </si>
+  <si>
+    <t>DARSSHINI P</t>
+  </si>
+  <si>
+    <t>Eathisha Fernandez G S</t>
+  </si>
+  <si>
+    <t>Fathina Begum B</t>
+  </si>
+  <si>
+    <t>Gurunethra.K</t>
+  </si>
+  <si>
+    <t>H Vikash</t>
+  </si>
+  <si>
+    <t>Harish Govind B</t>
+  </si>
+  <si>
+    <t>Harish K</t>
+  </si>
+  <si>
+    <t>Kaviarasi M</t>
+  </si>
+  <si>
+    <t>Krishnapriyabala JS</t>
+  </si>
+  <si>
+    <t>L VARSHA</t>
+  </si>
+  <si>
+    <t>Lakshana.A.N</t>
+  </si>
+  <si>
+    <t>Mahesh D</t>
+  </si>
+  <si>
+    <t>Meer Nadeem</t>
+  </si>
+  <si>
+    <t>Megaasri M</t>
+  </si>
+  <si>
+    <t>Mithul P</t>
+  </si>
+  <si>
+    <t>Mohamed Abbas S</t>
+  </si>
+  <si>
+    <t>Muthuraj R</t>
+  </si>
+  <si>
+    <t>Nikitha A</t>
+  </si>
+  <si>
+    <t>Nishanth V C</t>
+  </si>
+  <si>
+    <t>Parkavi Srinivasan</t>
+  </si>
+  <si>
+    <t>R.A.Karthiha</t>
+  </si>
+  <si>
+    <t>Rahul M A</t>
+  </si>
+  <si>
+    <t>Rohit.S.S</t>
+  </si>
+  <si>
+    <t>Rohith Kumar S</t>
+  </si>
+  <si>
+    <t>Sangita V</t>
+  </si>
+  <si>
+    <t>Sarvesh S</t>
+  </si>
+  <si>
+    <t>Shajith Ahamed S</t>
+  </si>
+  <si>
+    <t>Sherwin Richie J</t>
+  </si>
+  <si>
+    <t>SHREYA K P</t>
+  </si>
+  <si>
+    <t>Shri Varshini N</t>
+  </si>
+  <si>
+    <t>Siddharth Ramaswamy Ramkumar</t>
+  </si>
+  <si>
+    <t>Siddhartha Balaji</t>
+  </si>
+  <si>
+    <t>Srisanjay RD</t>
+  </si>
+  <si>
+    <t>Subin P</t>
+  </si>
+  <si>
+    <t>TAMILSELVAN S</t>
+  </si>
+  <si>
+    <t>Thiagarajan</t>
+  </si>
+  <si>
+    <t>Vijayalakshmi Radhakrishnan</t>
+  </si>
+  <si>
+    <t>Vineeth P</t>
+  </si>
+  <si>
+    <t>VISHNU PRASATH P</t>
+  </si>
+  <si>
+    <t>S.P.Deepakkumar</t>
+  </si>
+  <si>
+    <t>Andralyn Sweety H</t>
+  </si>
+  <si>
+    <t>Samyuktha Sowmyanarayanan</t>
+  </si>
+  <si>
+    <t>Nithin R</t>
+  </si>
+  <si>
+    <t>2/14/2008</t>
+  </si>
+  <si>
+    <t>12/31/2006</t>
+  </si>
+  <si>
+    <t>10/23/2006</t>
+  </si>
+  <si>
+    <t>11/25/2006</t>
+  </si>
+  <si>
+    <t>4/26/2008</t>
+  </si>
+  <si>
+    <t>12/16/2006</t>
+  </si>
+  <si>
+    <t>4/14/2008</t>
+  </si>
+  <si>
+    <t>2/17/2008</t>
+  </si>
+  <si>
+    <t>11/26/2007</t>
+  </si>
+  <si>
+    <t>2/18/2007</t>
+  </si>
+  <si>
+    <t>11/16/2006</t>
+  </si>
+  <si>
+    <t>9/29/2007</t>
+  </si>
+  <si>
+    <t>12/28/2007</t>
+  </si>
+  <si>
+    <t>10/17/2006</t>
+  </si>
+  <si>
+    <t>11/17/2007</t>
+  </si>
+  <si>
+    <t>10/22/2006</t>
+  </si>
+  <si>
+    <t>2/13/2008</t>
+  </si>
+  <si>
+    <t>3/24/2008</t>
+  </si>
+  <si>
+    <t>4/23/2007</t>
+  </si>
+  <si>
+    <t>12/27/2006</t>
+  </si>
+  <si>
+    <t>3/22/2008</t>
+  </si>
+  <si>
+    <t>6/21/2007</t>
+  </si>
+  <si>
+    <t>6/16/2007</t>
+  </si>
+  <si>
+    <t>5/14/2007</t>
+  </si>
+  <si>
+    <t>3/19/2007</t>
+  </si>
+  <si>
+    <t>9/24/2007</t>
+  </si>
+  <si>
+    <t>3/29/2007</t>
+  </si>
+  <si>
+    <t>11/30/2007</t>
+  </si>
+  <si>
+    <t>10/28/2007</t>
+  </si>
+  <si>
+    <t>2/20/2006</t>
+  </si>
+  <si>
+    <t>7/20/2007</t>
+  </si>
+  <si>
+    <t>10/15/2007</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +309,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -112,7 +343,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -135,44 +366,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -496,505 +743,775 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6">
-        <v>39666</v>
-      </c>
-      <c r="C4" s="12" t="s">
+      <c r="B4" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="12">
+        <v>39480</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="12">
+        <v>39203</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="13">
+        <v>39605</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="12">
+        <v>39454</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="13">
         <v>38935</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="6">
-        <v>38966</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="8"/>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="8"/>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="8"/>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="8"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="8"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="8"/>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="8"/>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="8"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="8"/>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="8"/>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="8"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="8"/>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="8"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="8"/>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="8"/>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="8"/>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="8"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="8"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="8"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="8"/>
+      <c r="C21" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" s="8"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="8"/>
+      <c r="A22" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="12">
+        <v>39243</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" s="8"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="8"/>
+      <c r="A23" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="8"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="8"/>
+      <c r="A24" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="12">
+        <v>38937</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="25" spans="1:3">
-      <c r="A25" s="8"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="8"/>
+      <c r="A25" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="26" spans="1:3">
-      <c r="A26" s="8"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="8"/>
+      <c r="A26" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="8"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="8"/>
+      <c r="A27" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="13">
+        <v>39237</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="28" spans="1:3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="8"/>
+      <c r="A28" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="12">
+        <v>39358</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="29" spans="1:3">
-      <c r="A29" s="8"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="8"/>
+      <c r="A29" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="30" spans="1:3">
-      <c r="A30" s="8"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="8"/>
+      <c r="A30" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="12">
+        <v>38056</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="31" spans="1:3">
-      <c r="A31" s="8"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="8"/>
+      <c r="A31" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="8"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="8"/>
+      <c r="A32" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="8"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="8"/>
+      <c r="A33" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="13">
+        <v>38875</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="8"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="8"/>
+      <c r="A34" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="8"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="8"/>
+      <c r="A35" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="36" spans="1:3">
-      <c r="A36" s="8"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="8"/>
+      <c r="A36" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="37" spans="1:3">
-      <c r="A37" s="8"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="8"/>
+      <c r="A37" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="38" spans="1:3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="8"/>
+      <c r="A38" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" s="8"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="8"/>
+      <c r="A39" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="13">
+        <v>39030</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" s="8"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="8"/>
+      <c r="A40" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="8"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="8"/>
+      <c r="A41" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="8"/>
+      <c r="A42" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="8"/>
-      <c r="B43" s="9"/>
-      <c r="C43" s="8"/>
+      <c r="A43" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="44" spans="1:3">
-      <c r="A44" s="8"/>
-      <c r="B44" s="9"/>
-      <c r="C44" s="8"/>
+      <c r="A44" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="45" spans="1:3">
-      <c r="A45" s="8"/>
-      <c r="B45" s="9"/>
-      <c r="C45" s="8"/>
+      <c r="A45" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B45" s="13">
+        <v>39124</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="46" spans="1:3">
-      <c r="A46" s="8"/>
-      <c r="B46" s="9"/>
-      <c r="C46" s="8"/>
+      <c r="A46" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="47" spans="1:3">
-      <c r="A47" s="8"/>
-      <c r="B47" s="9"/>
-      <c r="C47" s="8"/>
+      <c r="A47" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="13">
+        <v>39420</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="48" spans="1:3">
-      <c r="A48" s="8"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="8"/>
+      <c r="A48" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="49" spans="1:3">
-      <c r="A49" s="8"/>
-      <c r="B49" s="9"/>
-      <c r="C49" s="8"/>
+      <c r="A49" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="50" spans="1:3">
-      <c r="A50" s="8"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="8"/>
+      <c r="A50" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51" s="8"/>
-      <c r="B51" s="9"/>
-      <c r="C51" s="8"/>
+      <c r="A51" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52" s="8"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="8"/>
+      <c r="A52" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="53" spans="1:3">
-      <c r="A53" s="8"/>
-      <c r="B53" s="9"/>
-      <c r="C53" s="8"/>
+      <c r="A53" s="6"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="6"/>
     </row>
     <row r="54" spans="1:3">
-      <c r="A54" s="8"/>
-      <c r="B54" s="9"/>
-      <c r="C54" s="8"/>
+      <c r="A54" s="2"/>
+      <c r="B54" s="3"/>
+      <c r="C54" s="2"/>
     </row>
     <row r="55" spans="1:3">
-      <c r="A55" s="11"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
     </row>
     <row r="56" spans="1:3">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="11"/>
+      <c r="A56" s="4"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
     </row>
     <row r="57" spans="1:3">
-      <c r="A57" s="11"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
+      <c r="A57" s="4"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
     </row>
     <row r="58" spans="1:3">
-      <c r="A58" s="11"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
     </row>
     <row r="59" spans="1:3">
-      <c r="A59" s="11"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="11"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
     </row>
     <row r="60" spans="1:3">
-      <c r="A60" s="11"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="11"/>
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
     </row>
     <row r="61" spans="1:3">
-      <c r="A61" s="11"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
     </row>
     <row r="62" spans="1:3">
-      <c r="A62" s="11"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="11"/>
+      <c r="A62" s="4"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
     </row>
     <row r="63" spans="1:3">
-      <c r="A63" s="11"/>
-      <c r="B63" s="11"/>
-      <c r="C63" s="11"/>
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
     </row>
     <row r="64" spans="1:3">
-      <c r="A64" s="11"/>
-      <c r="B64" s="11"/>
-      <c r="C64" s="11"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
     </row>
     <row r="65" spans="1:3">
-      <c r="A65" s="11"/>
-      <c r="B65" s="11"/>
-      <c r="C65" s="11"/>
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
     </row>
     <row r="66" spans="1:3">
-      <c r="A66" s="11"/>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
     </row>
     <row r="67" spans="1:3">
-      <c r="A67" s="11"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="11"/>
+      <c r="A67" s="4"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
     </row>
     <row r="68" spans="1:3">
-      <c r="A68" s="11"/>
-      <c r="B68" s="11"/>
-      <c r="C68" s="11"/>
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
     </row>
     <row r="69" spans="1:3">
-      <c r="A69" s="11"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="11"/>
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
     </row>
     <row r="70" spans="1:3">
-      <c r="A70" s="11"/>
-      <c r="B70" s="11"/>
-      <c r="C70" s="11"/>
+      <c r="A70" s="4"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
     </row>
     <row r="71" spans="1:3">
-      <c r="A71" s="11"/>
-      <c r="B71" s="11"/>
-      <c r="C71" s="11"/>
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
     </row>
     <row r="72" spans="1:3">
-      <c r="A72" s="11"/>
-      <c r="B72" s="11"/>
-      <c r="C72" s="11"/>
+      <c r="A72" s="4"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
     </row>
     <row r="73" spans="1:3">
-      <c r="A73" s="11"/>
-      <c r="B73" s="11"/>
-      <c r="C73" s="11"/>
+      <c r="A73" s="4"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
     </row>
     <row r="74" spans="1:3">
-      <c r="A74" s="11"/>
-      <c r="B74" s="11"/>
-      <c r="C74" s="11"/>
+      <c r="A74" s="4"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
     </row>
     <row r="75" spans="1:3">
-      <c r="A75" s="11"/>
-      <c r="B75" s="11"/>
-      <c r="C75" s="11"/>
+      <c r="A75" s="4"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
     </row>
     <row r="76" spans="1:3">
-      <c r="A76" s="11"/>
-      <c r="B76" s="11"/>
-      <c r="C76" s="11"/>
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
     </row>
     <row r="77" spans="1:3">
-      <c r="A77" s="11"/>
-      <c r="B77" s="11"/>
-      <c r="C77" s="11"/>
+      <c r="A77" s="4"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
     </row>
     <row r="78" spans="1:3">
-      <c r="A78" s="11"/>
-      <c r="B78" s="11"/>
-      <c r="C78" s="11"/>
+      <c r="A78" s="4"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
     </row>
     <row r="79" spans="1:3">
-      <c r="A79" s="11"/>
-      <c r="B79" s="11"/>
-      <c r="C79" s="11"/>
+      <c r="A79" s="4"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
     </row>
     <row r="80" spans="1:3">
-      <c r="A80" s="11"/>
-      <c r="B80" s="11"/>
-      <c r="C80" s="11"/>
+      <c r="A80" s="4"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
     </row>
     <row r="81" spans="1:3">
-      <c r="A81" s="11"/>
-      <c r="B81" s="11"/>
-      <c r="C81" s="11"/>
+      <c r="A81" s="4"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
     </row>
     <row r="82" spans="1:3">
-      <c r="A82" s="11"/>
-      <c r="B82" s="11"/>
-      <c r="C82" s="11"/>
+      <c r="A82" s="4"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
     </row>
     <row r="83" spans="1:3">
-      <c r="A83" s="11"/>
-      <c r="B83" s="11"/>
-      <c r="C83" s="11"/>
+      <c r="A83" s="4"/>
+      <c r="B83" s="4"/>
+      <c r="C83" s="4"/>
     </row>
     <row r="84" spans="1:3">
-      <c r="A84" s="11"/>
-      <c r="B84" s="11"/>
-      <c r="C84" s="11"/>
+      <c r="A84" s="4"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
     </row>
     <row r="85" spans="1:3">
-      <c r="A85" s="11"/>
-      <c r="B85" s="11"/>
-      <c r="C85" s="11"/>
+      <c r="A85" s="4"/>
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
     </row>
     <row r="86" spans="1:3">
-      <c r="A86" s="11"/>
-      <c r="B86" s="11"/>
-      <c r="C86" s="11"/>
+      <c r="A86" s="4"/>
+      <c r="B86" s="4"/>
+      <c r="C86" s="4"/>
     </row>
     <row r="87" spans="1:3">
-      <c r="A87" s="11"/>
-      <c r="B87" s="11"/>
-      <c r="C87" s="11"/>
+      <c r="A87" s="4"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
     </row>
     <row r="88" spans="1:3">
-      <c r="A88" s="11"/>
-      <c r="B88" s="11"/>
-      <c r="C88" s="11"/>
+      <c r="A88" s="4"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
     </row>
     <row r="89" spans="1:3">
-      <c r="A89" s="11"/>
-      <c r="B89" s="11"/>
-      <c r="C89" s="11"/>
+      <c r="A89" s="4"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
     </row>
     <row r="90" spans="1:3">
-      <c r="A90" s="11"/>
-      <c r="B90" s="11"/>
-      <c r="C90" s="11"/>
+      <c r="A90" s="4"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
     </row>
     <row r="91" spans="1:3">
-      <c r="A91" s="11"/>
-      <c r="B91" s="11"/>
-      <c r="C91" s="11"/>
+      <c r="A91" s="4"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
     </row>
     <row r="92" spans="1:3">
-      <c r="A92" s="11"/>
-      <c r="B92" s="11"/>
-      <c r="C92" s="11"/>
+      <c r="A92" s="4"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
     </row>
     <row r="93" spans="1:3">
-      <c r="A93" s="11"/>
-      <c r="B93" s="11"/>
-      <c r="C93" s="11"/>
+      <c r="A93" s="4"/>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
     </row>
     <row r="94" spans="1:3">
-      <c r="A94" s="11"/>
-      <c r="B94" s="11"/>
-      <c r="C94" s="11"/>
+      <c r="A94" s="4"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1004,6 +1521,7 @@
     <hyperlink ref="C5" r:id="rId4"/>
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
+    <hyperlink ref="C8:C52" r:id="rId7" display="alfredsam427@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Support Excel date cells and MM/DD/YYYY / MM-DD-YYYY strings in DOB parsing, and update bdays.xlsx
</commit_message>
<xml_diff>
--- a/bdays.xlsx
+++ b/bdays.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="89">
   <si>
     <t>Name</t>
   </si>
@@ -343,7 +343,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -379,6 +379,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -406,19 +421,19 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -723,15 +738,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="37.7109375" customWidth="1"/>
     <col min="2" max="2" width="27.7109375" customWidth="1"/>
     <col min="3" max="3" width="61.140625" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -742,19 +758,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" ht="15.75" thickBot="1">
       <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A3" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="11" t="s">
@@ -764,19 +780,19 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="11" t="s">
@@ -786,19 +802,19 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" ht="15.75" thickBot="1">
       <c r="A6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>59</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="11" t="s">
@@ -808,19 +824,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" ht="15.75" thickBot="1">
       <c r="A8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A9" s="9" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="11" t="s">
@@ -830,7 +846,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" ht="15.75" thickBot="1">
       <c r="A10" s="8" t="s">
         <v>15</v>
       </c>
@@ -841,8 +857,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A11" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="11" t="s">
@@ -852,19 +868,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" ht="15.75" thickBot="1">
       <c r="A12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>64</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A13" s="9" t="s">
         <v>18</v>
       </c>
       <c r="B13" s="11" t="s">
@@ -874,7 +890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" ht="15.75" thickBot="1">
       <c r="A14" s="8" t="s">
         <v>19</v>
       </c>
@@ -885,8 +901,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A15" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="13">
@@ -896,19 +912,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" ht="15.75" thickBot="1">
       <c r="A16" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A17" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B17" s="11" t="s">
@@ -918,7 +934,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" ht="15.75" thickBot="1">
       <c r="A18" s="8" t="s">
         <v>23</v>
       </c>
@@ -929,8 +945,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A19" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B19" s="11" t="s">
@@ -940,19 +956,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" ht="15.75" thickBot="1">
       <c r="A20" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="10" t="s">
         <v>69</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A21" s="9" t="s">
         <v>26</v>
       </c>
       <c r="B21" s="13">
@@ -962,7 +978,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" ht="15.75" thickBot="1">
       <c r="A22" s="8" t="s">
         <v>27</v>
       </c>
@@ -973,8 +989,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A23" s="9" t="s">
         <v>28</v>
       </c>
       <c r="B23" s="11" t="s">
@@ -984,7 +1000,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" ht="15.75" thickBot="1">
       <c r="A24" s="8" t="s">
         <v>29</v>
       </c>
@@ -995,8 +1011,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A25" s="9" t="s">
         <v>30</v>
       </c>
       <c r="B25" s="11" t="s">
@@ -1006,312 +1022,306 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>71</v>
+    <row r="26" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A26" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="13">
+        <v>39237</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="13">
-        <v>39237</v>
+    <row r="27" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A27" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="12">
+        <v>39358</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="12">
-        <v>39358</v>
+    <row r="28" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A28" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>72</v>
+    <row r="29" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A29" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="12">
+        <v>38056</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" s="12">
-        <v>38056</v>
+    <row r="30" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A30" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>73</v>
+    <row r="31" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A31" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>74</v>
+    <row r="32" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A32" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="13">
+        <v>38875</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="13">
-        <v>38875</v>
+    <row r="33" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A33" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>75</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>75</v>
+    <row r="34" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A34" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>76</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="11" t="s">
+    <row r="35" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A35" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A36" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>77</v>
-      </c>
       <c r="C36" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B37" s="11" t="s">
-        <v>76</v>
+    <row r="37" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A37" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>78</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>78</v>
+    <row r="38" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A38" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="13">
+        <v>39030</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B39" s="13">
-        <v>39030</v>
+    <row r="39" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A39" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>79</v>
+    <row r="40" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A40" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B41" s="11" t="s">
-        <v>80</v>
+    <row r="41" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A41" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
-      <c r="A42" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B42" s="9" t="s">
-        <v>81</v>
+    <row r="42" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A42" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
-      <c r="A43" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>82</v>
+    <row r="43" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A43" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
-      <c r="A44" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>83</v>
+    <row r="44" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A44" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44" s="13">
+        <v>39124</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
-      <c r="A45" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B45" s="13">
-        <v>39124</v>
+    <row r="45" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A45" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
-      <c r="A46" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>84</v>
+    <row r="46" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A46" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46" s="13">
+        <v>39420</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
-      <c r="A47" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B47" s="13">
-        <v>39420</v>
+    <row r="47" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A47" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
-      <c r="A48" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>85</v>
+    <row r="48" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A48" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>86</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
-      <c r="A49" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B49" s="11" t="s">
-        <v>86</v>
+    <row r="49" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A49" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
-      <c r="A50" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>87</v>
+    <row r="50" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A50" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
-      <c r="A51" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B51" s="11" t="s">
-        <v>67</v>
+    <row r="51" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A51" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A52" s="6"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="6"/>
     </row>
     <row r="53" spans="1:3">
-      <c r="A53" s="6"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="6"/>
+      <c r="A53" s="2"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="2"/>
     </row>
     <row r="54" spans="1:3">
-      <c r="A54" s="2"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="2"/>
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="4"/>
@@ -1507,11 +1517,6 @@
       <c r="A93" s="4"/>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94" s="4"/>
-      <c r="B94" s="4"/>
-      <c r="C94" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1521,7 +1526,7 @@
     <hyperlink ref="C5" r:id="rId4"/>
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
-    <hyperlink ref="C8:C52" r:id="rId7" display="alfredsam427@gmail.com"/>
+    <hyperlink ref="C8:C51" r:id="rId7" display="alfredsam427@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>